<commit_message>
publish: 63a8bfb39228e78a795caf952d8814f7ce614317 (run 30530772720)
</commit_message>
<xml_diff>
--- a/snomed-mappings.xlsx
+++ b/snomed-mappings.xlsx
@@ -295,7 +295,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t xml:space="preserve">VERIFIED</t>
+          <t xml:space="preserve">待覆核</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -343,7 +343,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t xml:space="preserve">VERIFIED</t>
+          <t xml:space="preserve">待覆核</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -395,7 +395,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t xml:space="preserve">VERIFIED</t>
+          <t xml:space="preserve">待覆核</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -447,7 +447,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t xml:space="preserve">VERIFIED</t>
+          <t xml:space="preserve">待覆核</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -499,7 +499,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t xml:space="preserve">VERIFIED</t>
+          <t xml:space="preserve">待覆核</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -547,7 +547,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t xml:space="preserve">VERIFIED</t>
+          <t xml:space="preserve">待覆核</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -599,7 +599,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t xml:space="preserve">VERIFIED</t>
+          <t xml:space="preserve">待覆核</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -651,7 +651,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t xml:space="preserve">VERIFIED</t>
+          <t xml:space="preserve">待覆核</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -703,7 +703,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t xml:space="preserve">VERIFIED</t>
+          <t xml:space="preserve">待覆核</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -755,7 +755,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t xml:space="preserve">VERIFIED</t>
+          <t xml:space="preserve">待覆核</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -807,7 +807,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t xml:space="preserve">VERIFIED</t>
+          <t xml:space="preserve">待覆核</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -859,7 +859,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t xml:space="preserve">VERIFIED</t>
+          <t xml:space="preserve">待覆核</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -911,7 +911,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t xml:space="preserve">VERIFIED</t>
+          <t xml:space="preserve">待覆核</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -963,7 +963,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t xml:space="preserve">VERIFIED</t>
+          <t xml:space="preserve">待覆核</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1015,7 +1015,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t xml:space="preserve">VERIFIED</t>
+          <t xml:space="preserve">待覆核</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1067,7 +1067,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t xml:space="preserve">VERIFIED</t>
+          <t xml:space="preserve">待覆核</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1119,7 +1119,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t xml:space="preserve">VERIFIED</t>
+          <t xml:space="preserve">待覆核</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1171,7 +1171,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t xml:space="preserve">VERIFIED</t>
+          <t xml:space="preserve">待覆核</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1223,7 +1223,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t xml:space="preserve">VERIFIED</t>
+          <t xml:space="preserve">待覆核</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1275,7 +1275,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t xml:space="preserve">VERIFIED</t>
+          <t xml:space="preserve">待覆核</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1327,7 +1327,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t xml:space="preserve">VERIFIED</t>
+          <t xml:space="preserve">待覆核</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -1379,7 +1379,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t xml:space="preserve">VERIFIED</t>
+          <t xml:space="preserve">待覆核</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -1431,7 +1431,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t xml:space="preserve">VERIFIED</t>
+          <t xml:space="preserve">待覆核</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -1483,7 +1483,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t xml:space="preserve">VERIFIED</t>
+          <t xml:space="preserve">待覆核</t>
         </is>
       </c>
       <c r="I25"/>
@@ -1531,7 +1531,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t xml:space="preserve">VERIFIED</t>
+          <t xml:space="preserve">待覆核</t>
         </is>
       </c>
       <c r="I26"/>
@@ -1579,7 +1579,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t xml:space="preserve">VERIFIED</t>
+          <t xml:space="preserve">待覆核</t>
         </is>
       </c>
       <c r="I27"/>
@@ -1623,7 +1623,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t xml:space="preserve">VERIFIED</t>
+          <t xml:space="preserve">待覆核</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -1655,7 +1655,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t xml:space="preserve">73708-3</t>
+          <t xml:space="preserve">(-確定無合適碼)</t>
         </is>
       </c>
       <c r="E29"/>
@@ -1671,7 +1671,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t xml:space="preserve">VERIFIED</t>
+          <t xml:space="preserve">待覆核</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -1719,7 +1719,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t xml:space="preserve">VERIFIED</t>
+          <t xml:space="preserve">待覆核</t>
         </is>
       </c>
       <c r="I30"/>
@@ -1767,7 +1767,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t xml:space="preserve">VERIFIED</t>
+          <t xml:space="preserve">待覆核</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -1815,7 +1815,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t xml:space="preserve">VERIFIED</t>
+          <t xml:space="preserve">待覆核</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -1847,7 +1847,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t xml:space="preserve">79880-1</t>
+          <t xml:space="preserve">98497-1</t>
         </is>
       </c>
       <c r="E33"/>
@@ -1863,7 +1863,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t xml:space="preserve">VERIFIED</t>
+          <t xml:space="preserve">待覆核</t>
         </is>
       </c>
       <c r="I33"/>
@@ -1907,7 +1907,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t xml:space="preserve">VERIFIED</t>
+          <t xml:space="preserve">待覆核</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">

</xml_diff>